<commit_message>
Ergebnis manuell: Mexiko 2:0 Südafrika
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -470,7 +470,11 @@
           <t>11.06.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,7 +497,6 @@
           <t>12.06.</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -516,7 +519,6 @@
           <t>18.06.</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -539,7 +541,6 @@
           <t>19.06.</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -562,7 +563,6 @@
           <t>25.06.</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -585,7 +585,6 @@
           <t>25.06.</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -608,7 +607,6 @@
           <t>12.06.</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -631,7 +629,6 @@
           <t>13.06.</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -654,7 +651,6 @@
           <t>18.06.</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -677,7 +673,6 @@
           <t>19.06.</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -700,7 +695,6 @@
           <t>24.06.</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -723,7 +717,6 @@
           <t>24.06.</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -746,7 +739,6 @@
           <t>14.06.</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -769,7 +761,6 @@
           <t>14.06.</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -792,7 +783,6 @@
           <t>20.06.</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -815,7 +805,6 @@
           <t>20.06.</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -838,7 +827,6 @@
           <t>25.06.</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -861,7 +849,6 @@
           <t>25.06.</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -884,7 +871,6 @@
           <t>13.06.</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -907,7 +893,6 @@
           <t>14.06.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -930,7 +915,6 @@
           <t>19.06.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -953,7 +937,6 @@
           <t>20.06.</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -976,7 +959,6 @@
           <t>26.06.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -999,7 +981,6 @@
           <t>26.06.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1022,7 +1003,6 @@
           <t>14.06.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1045,7 +1025,6 @@
           <t>15.06.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1068,7 +1047,6 @@
           <t>20.06.</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1091,7 +1069,6 @@
           <t>21.06.</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1114,7 +1091,6 @@
           <t>25.06.</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1137,7 +1113,6 @@
           <t>25.06.</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1160,7 +1135,6 @@
           <t>14.06.</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1183,7 +1157,6 @@
           <t>15.06.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1206,7 +1179,6 @@
           <t>20.06.</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1229,7 +1201,6 @@
           <t>21.06.</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1252,7 +1223,6 @@
           <t>26.06.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1275,7 +1245,6 @@
           <t>26.06.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1298,7 +1267,6 @@
           <t>15.06.</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1321,7 +1289,6 @@
           <t>16.06.</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1344,7 +1311,6 @@
           <t>21.06.</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1367,7 +1333,6 @@
           <t>22.06.</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1390,7 +1355,6 @@
           <t>27.06.</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1413,7 +1377,6 @@
           <t>27.06.</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1436,7 +1399,6 @@
           <t>15.06.</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1459,7 +1421,6 @@
           <t>16.06.</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1482,7 +1443,6 @@
           <t>21.06.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1505,7 +1465,6 @@
           <t>22.06.</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1528,7 +1487,6 @@
           <t>27.06.</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1551,7 +1509,6 @@
           <t>27.06.</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1574,7 +1531,6 @@
           <t>16.06.</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1597,7 +1553,6 @@
           <t>17.06.</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1620,7 +1575,6 @@
           <t>22.06.</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1643,7 +1597,6 @@
           <t>23.06.</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1666,7 +1619,6 @@
           <t>26.06.</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1689,7 +1641,6 @@
           <t>26.06.</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1712,7 +1663,6 @@
           <t>17.06.</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1735,7 +1685,6 @@
           <t>17.06.</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1758,7 +1707,6 @@
           <t>22.06.</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1781,7 +1729,6 @@
           <t>23.06.</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1804,7 +1751,6 @@
           <t>28.06.</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1827,7 +1773,6 @@
           <t>28.06.</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1850,7 +1795,6 @@
           <t>17.06.</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1873,7 +1817,6 @@
           <t>18.06.</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1896,7 +1839,6 @@
           <t>23.06.</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1919,7 +1861,6 @@
           <t>24.06.</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1942,7 +1883,6 @@
           <t>28.06.</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1965,7 +1905,6 @@
           <t>28.06.</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1988,7 +1927,6 @@
           <t>17.06.</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2011,7 +1949,6 @@
           <t>18.06.</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2034,7 +1971,6 @@
           <t>23.06.</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2057,7 +1993,6 @@
           <t>24.06.</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2080,7 +2015,6 @@
           <t>27.06.</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2103,7 +2037,6 @@
           <t>27.06.</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Ergebnis: Südkorea 2:1 Tschechien; Match-Fenster auf 6h erhöht
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -497,6 +497,11 @@
           <t>12.06.</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">

</xml_diff>

<commit_message>
ESPN API: sofortige Ergebnisse ohne API-Key, kein Verzögerungsproblem mehr
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -524,6 +524,7 @@
           <t>18.06.</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -546,6 +547,7 @@
           <t>19.06.</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -568,6 +570,7 @@
           <t>25.06.</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -590,6 +593,7 @@
           <t>25.06.</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -612,6 +616,7 @@
           <t>12.06.</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -634,6 +639,7 @@
           <t>13.06.</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -656,6 +662,7 @@
           <t>18.06.</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -678,6 +685,7 @@
           <t>19.06.</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -700,6 +708,7 @@
           <t>24.06.</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -722,6 +731,7 @@
           <t>24.06.</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -744,6 +754,7 @@
           <t>14.06.</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -766,6 +777,7 @@
           <t>14.06.</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -788,6 +800,7 @@
           <t>20.06.</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -810,6 +823,7 @@
           <t>20.06.</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -832,6 +846,7 @@
           <t>25.06.</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -854,6 +869,7 @@
           <t>25.06.</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -876,6 +892,7 @@
           <t>13.06.</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -898,6 +915,7 @@
           <t>14.06.</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -920,6 +938,7 @@
           <t>19.06.</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -942,6 +961,7 @@
           <t>20.06.</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -964,6 +984,7 @@
           <t>26.06.</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -986,6 +1007,7 @@
           <t>26.06.</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1008,6 +1030,7 @@
           <t>14.06.</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1030,6 +1053,7 @@
           <t>15.06.</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1052,6 +1076,7 @@
           <t>20.06.</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1074,6 +1099,7 @@
           <t>21.06.</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1096,6 +1122,7 @@
           <t>25.06.</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1118,6 +1145,7 @@
           <t>25.06.</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1140,6 +1168,7 @@
           <t>14.06.</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1162,6 +1191,7 @@
           <t>15.06.</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1184,6 +1214,7 @@
           <t>20.06.</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1206,6 +1237,7 @@
           <t>21.06.</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1228,6 +1260,7 @@
           <t>26.06.</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1250,6 +1283,7 @@
           <t>26.06.</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1272,6 +1306,7 @@
           <t>15.06.</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1294,6 +1329,7 @@
           <t>16.06.</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1316,6 +1352,7 @@
           <t>21.06.</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1338,6 +1375,7 @@
           <t>22.06.</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1360,6 +1398,7 @@
           <t>27.06.</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1382,6 +1421,7 @@
           <t>27.06.</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1404,6 +1444,7 @@
           <t>15.06.</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1426,6 +1467,7 @@
           <t>16.06.</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1448,6 +1490,7 @@
           <t>21.06.</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1470,6 +1513,7 @@
           <t>22.06.</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1492,6 +1536,7 @@
           <t>27.06.</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1514,6 +1559,7 @@
           <t>27.06.</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1536,6 +1582,7 @@
           <t>16.06.</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1558,6 +1605,7 @@
           <t>17.06.</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1580,6 +1628,7 @@
           <t>22.06.</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1602,6 +1651,7 @@
           <t>23.06.</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1624,6 +1674,7 @@
           <t>26.06.</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1646,6 +1697,7 @@
           <t>26.06.</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1668,6 +1720,7 @@
           <t>17.06.</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1690,6 +1743,7 @@
           <t>17.06.</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1712,6 +1766,7 @@
           <t>22.06.</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1734,6 +1789,7 @@
           <t>23.06.</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1756,6 +1812,7 @@
           <t>28.06.</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1778,6 +1835,7 @@
           <t>28.06.</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1800,6 +1858,7 @@
           <t>17.06.</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1822,6 +1881,7 @@
           <t>18.06.</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1844,6 +1904,7 @@
           <t>23.06.</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1866,6 +1927,7 @@
           <t>24.06.</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1888,6 +1950,7 @@
           <t>28.06.</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1910,6 +1973,7 @@
           <t>28.06.</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1932,6 +1996,7 @@
           <t>17.06.</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1954,6 +2019,7 @@
           <t>18.06.</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1976,6 +2042,7 @@
           <t>23.06.</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1998,6 +2065,7 @@
           <t>24.06.</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2020,6 +2088,7 @@
           <t>27.06.</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2042,6 +2111,7 @@
           <t>27.06.</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix: GQ auch ohne API-Abruf berechnen wenn Gruppenphase abgeschlossen
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -14,6 +14,7 @@
     <sheet name="HF" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="F" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="WM" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="GQ" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2552,4 +2553,350 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mexiko</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Südafrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Schweiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kanada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Australien</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Niederlande</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ägypten</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kap Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Norwegen</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Österreich</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Schweden</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bosnien-Herzegowina</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Algerien</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: S16-Sieger korrekt parsen, KO-Phase automatisch erkennen
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -8,13 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Gruppenphase" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="S16" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="S8" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="VF" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="HF" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="WM" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="GQ" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="GQ" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="S16" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="S8" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="VF" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="HF" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="F" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="WM" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2405,7 +2405,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2417,6 +2417,326 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mexiko</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Südafrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Schweiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Kanada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Australien</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Niederlande</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ägypten</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kap Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Norwegen</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Österreich</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Schweden</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bosnien-Herzegowina</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Algerien</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
@@ -2431,7 +2751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2443,6 +2763,46 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kanada</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2576,326 +2936,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Mexiko</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Südafrika</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Schweiz</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Kanada</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Brasilien</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Australien</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Elfenbeinküste</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Niederlande</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Belgien</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Ägypten</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Spanien</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Kap Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Norwegen</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Argentinien</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Österreich</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Kolumbien</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Kroatien</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Schweden</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Bosnien-Herzegowina</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Algerien</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: KO-Runden Datum-Mapping, S8 einpflegen, Default-Tab dynamisch
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -2751,7 +2751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2913,16 +2913,6 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>Argentinien</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Kolumbien</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2949,6 +2939,36 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: S16 komplett (16/16), S8 Marokko+Frankreich eingetragen
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -2751,7 +2751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2913,6 +2913,16 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>Argentinien</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
         </is>
       </c>
     </row>
@@ -2927,7 +2937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2948,7 +2958,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Kolumbien</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
@@ -2957,16 +2967,6 @@
         <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
         <is>
           <t>Frankreich</t>
         </is>

</xml_diff>

<commit_message>
HF/P3: Frankreich als P3-Teilnehmer, Default-Tab auf Finale, P3-Sieger-Logik
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -13,8 +13,10 @@
     <sheet name="S8" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="VF" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="HF" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="F" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="WM" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="P3" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="P3_participants" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="F" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="WM" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2399,6 +2401,32 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3171,6 +3199,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Fix: F aus HF-Siegern, P3 aus HF-Verlierern ableiten; Spanien im Finale, Frankreich P3
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -3173,7 +3173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3185,6 +3185,16 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>Team</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Frankreich</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3250,6 +3260,16 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
P3: Frankreich nur als Teilnehmer, Sieger erst nach Spiel; Scoring-Zeile hinzugefügt
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -3173,7 +3173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3185,16 +3185,6 @@
       <c r="B1" t="inlineStr">
         <is>
           <t>Team</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix: Finale Spanien vs Argentinien, P3 Frankreich vs England
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -3255,7 +3255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3280,6 +3280,16 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
WM beendet: Cron deaktiviert, England P3-Sieger, Spanien WM, WM-Tab Default
</commit_message>
<xml_diff>
--- a/Ergebnisse.xlsx
+++ b/Ergebnisse.xlsx
@@ -3214,30 +3214,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Frankreich</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
           <t>England</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-    </row>
+    <row r="3"/>
+    <row r="4"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>